<commit_message>
chore: persist Strategy B paper state
</commit_message>
<xml_diff>
--- a/data/strategy_b_paper_history.xlsx
+++ b/data/strategy_b_paper_history.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CONDITIONS'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DAILY_SUMMARY'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PERFORMANCE'!$A$1:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SYSTEM_LOG'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SYSTEM_LOG'!$A$1:$D$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -803,7 +803,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-20T13:33:22.884427+00:00</t>
+          <t>2026-10-21T04:35:20.589665+00:00</t>
         </is>
       </c>
     </row>
@@ -819,13 +819,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -850,8 +850,624 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:37.703325+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ADANIENT: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:39.200021+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:39.926736+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ASIANPAINT: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:40.720482+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AXISBANK: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:41.446307+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:43.764156+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BEL: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:46.062603+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>COALINDIA: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:49.909442+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>HCLTECH: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:52.921048+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>HINDALCO: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:53.636557+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>HINDUNILVR: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:55.184887+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>INDUSINDBK: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:34:55.940950+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>INFY: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:01.546760+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>JSWSTEEL: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:03.036931+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>LT: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:07.594009+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ONGC: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:08.315009+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>POWERGRID: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:09.039293+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>RELIANCE: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:09.762920+00:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SBILIFE: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:11.151615+00:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SBIN: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:12.657139+00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SUNPHARMA: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:13.382530+00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>TATACONSUM: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:14.110708+00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>TATASTEEL: SmartAPI returned no candle data for token 3499: Too many requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:14.840292+00:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TCS: SmartAPI returned no candle data for token 11536: Too many requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:15.563337+00:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>TECHM: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:16.283455+00:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>TITAN: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:17.012437+00:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>TRENT: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:18.548818+00:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>WIPRO: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-21T04:35:19.276365+00:00</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TMPV: Couldn't parse the JSON response received from the server: b'Access denied because of exceeding access rate'</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:D29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: persist paper scanner outputs
</commit_message>
<xml_diff>
--- a/data/strategy_b_paper_history.xlsx
+++ b/data/strategy_b_paper_history.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CONDITIONS'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DAILY_SUMMARY'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PERFORMANCE'!$A$1:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SYSTEM_LOG'!$A$1:$D$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SYSTEM_LOG'!$A$1:$D$275</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -803,7 +803,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-21T18:22:23.892342+00:00</t>
+          <t>2026-10-21T18:31:08.765420+00:00</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D178"/>
+  <dimension ref="A1:D275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4744,8 +4744,2142 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:00.831221+00:00</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>TATAINVEST: SmartAPI returned no candle data for token 1621: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:01.523811+00:00</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>TATAPOWER: SmartAPI returned no candle data for token 3426: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:02.275360+00:00</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>TCS: SmartAPI returned no candle data for token 11536: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:02.960037+00:00</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>TDPOWERSYS: SmartAPI returned no candle data for token 25178: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:03.641439+00:00</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>TECHNOE: SmartAPI returned no candle data for token 6445: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:04.333677+00:00</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>TEGA: SmartAPI returned no candle data for token 7105: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:05.030464+00:00</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>TEJASNET: SmartAPI returned no candle data for token 21131: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:05.718661+00:00</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>TIINDIA: SmartAPI returned no candle data for token 312: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:06.421067+00:00</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>TIMKEN: SmartAPI returned no candle data for token 14198: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:07.107925+00:00</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>TMCV: SmartAPI returned no candle data for token 759782: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:07.789524+00:00</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>TMPV: SmartAPI returned no candle data for token 3456: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:08.479523+00:00</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>TRITURBINE: SmartAPI returned no candle data for token 25584: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:09.240085+00:00</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>USHAMART: SmartAPI returned no candle data for token 8840: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:09.954498+00:00</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>VAML: SmartAPI returned no candle data for token 750174: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:10.635945+00:00</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>VBL: SmartAPI returned no candle data for token 18921: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:11.352709+00:00</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>VOLTAS: SmartAPI returned no candle data for token 3718: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:12.033532+00:00</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>WELCORP: SmartAPI returned no candle data for token 11821: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:12.737971+00:00</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV: SmartAPI returned no candle data for token 11253: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:13.431222+00:00</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>WHIRLPOOL: SmartAPI returned no candle data for token 18011: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:14.113740+00:00</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>ZENSARTECH: SmartAPI returned no candle data for token 1076: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:14.805636+00:00</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>ZENTEC: SmartAPI returned no candle data for token 7508: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:15.520617+00:00</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>ZFCVINDIA: SmartAPI returned no candle data for token 16915: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:16.242501+00:00</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>AARTIIND: SmartAPI returned no candle data for token 7: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:16.964541+00:00</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>ABCAPITAL: SmartAPI returned no candle data for token 21614: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:17.663510+00:00</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>ACC: SmartAPI returned no candle data for token 22: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:18.378546+00:00</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>ACE: SmartAPI returned no candle data for token 13587: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:19.063133+00:00</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>ACMESOLAR: SmartAPI returned no candle data for token 27061: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:19.792134+00:00</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>ADANIGREEN: SmartAPI returned no candle data for token 3563: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:20.477811+00:00</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>ADANIPORTS: SmartAPI returned no candle data for token 15083: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:21.179903+00:00</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>AETHER: SmartAPI returned no candle data for token 9810: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:21.869997+00:00</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>AFCONS: SmartAPI returned no candle data for token 25977: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:22.563960+00:00</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>AIIL: SmartAPI returned no candle data for token 23553: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:23.333636+00:00</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>AMBUJACEM: SmartAPI returned no candle data for token 1270: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:24.032516+00:00</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>ANANDRATHI: SmartAPI returned no candle data for token 7145: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:24.751034+00:00</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>APLAPOLLO: SmartAPI returned no candle data for token 25780: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:25.451555+00:00</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>APOLLOTYRE: SmartAPI returned no candle data for token 163: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:26.145563+00:00</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>ARE&amp;M: SmartAPI returned no candle data for token 100: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:26.827769+00:00</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>ASIANPAINT: SmartAPI returned no candle data for token 236: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:27.545131+00:00</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>ASTERDM: SmartAPI returned no candle data for token 1508: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:28.268590+00:00</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>ASTRAL: SmartAPI returned no candle data for token 14418: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:28.957163+00:00</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>ATHERENERG: SmartAPI returned no candle data for token 757645: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:29.649179+00:00</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>AUBANK: SmartAPI returned no candle data for token 21238: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:30.341748+00:00</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>AUROPHARMA: SmartAPI returned no candle data for token 275: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:31.031593+00:00</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>AVANTIFEED: SmartAPI returned no candle data for token 7936: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:31.726093+00:00</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>AXISBANK: SmartAPI returned no candle data for token 5900: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:32.414549+00:00</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>AZAD: SmartAPI returned no candle data for token 20905: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:33.099135+00:00</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV: SmartAPI returned no candle data for token 16675: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:33.788022+00:00</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>BAJFINANCE: SmartAPI returned no candle data for token 317: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:34.483672+00:00</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>BALKRISIND: SmartAPI returned no candle data for token 335: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:35.207326+00:00</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>BALRAMCHIN: SmartAPI returned no candle data for token 341: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:35.891370+00:00</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>BANKBARODA: SmartAPI returned no candle data for token 4668: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:36.628925+00:00</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>BBOX: SmartAPI returned no candle data for token 3435: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:37.340746+00:00</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>BEL: SmartAPI returned no candle data for token 383: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:38.027274+00:00</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>BERGEPAINT: SmartAPI returned no candle data for token 404: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:38.719867+00:00</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>BIOCON: SmartAPI returned no candle data for token 11373: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:39.415072+00:00</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>BLS: SmartAPI returned no candle data for token 17279: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:40.100590+00:00</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>BRIGADE: SmartAPI returned no candle data for token 15184: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:40.791154+00:00</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>BSOFT: SmartAPI returned no candle data for token 6994: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:41.474571+00:00</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>CAMS: SmartAPI returned no candle data for token 342: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:42.229363+00:00</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>CAPLIPOINT: SmartAPI returned no candle data for token 3906: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:42.949634+00:00</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>CEMPRO: SmartAPI returned no candle data for token 5622: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:43.674813+00:00</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>CGCL: SmartAPI returned no candle data for token 20329: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:44.382913+00:00</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>CHAMBLFERT: SmartAPI returned no candle data for token 637: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:45.161769+00:00</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>CHENNPETRO: SmartAPI returned no candle data for token 2049: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:45.857729+00:00</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>CLEANMAX: SmartAPI returned no candle data for token 760183: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:46.592120+00:00</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>COALINDIA: SmartAPI returned no candle data for token 20374: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:47.354651+00:00</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>COFORGE: SmartAPI returned no candle data for token 11543: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:48.047993+00:00</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>CONCORDBIO: SmartAPI returned no candle data for token 18060: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:48.807739+00:00</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>CREDITACC: SmartAPI returned no candle data for token 4421: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:49.514508+00:00</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>CUPID: SmartAPI returned no candle data for token 18520: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:50.235478+00:00</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>CYIENT: SmartAPI returned no candle data for token 5748: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:50.981527+00:00</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>DALBHARAT: SmartAPI returned no candle data for token 8075: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:51.705694+00:00</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>DELHIVERY: SmartAPI returned no candle data for token 9599: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:52.425670+00:00</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>EIHOTEL: SmartAPI returned no candle data for token 919: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:53.116075+00:00</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>ELGIEQUIP: SmartAPI returned no candle data for token 937: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:53.842621+00:00</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>EMAMILTD: SmartAPI returned no candle data for token 13517: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:54.561884+00:00</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>EMCURE: SmartAPI returned no candle data for token 24398: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:55.242093+00:00</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>EMMVEE: SmartAPI returned no candle data for token 759728: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:55.994597+00:00</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>ENGINERSIN: SmartAPI returned no candle data for token 4907: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:56.676599+00:00</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>ESCORTS: SmartAPI returned no candle data for token 958: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:57.389416+00:00</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>FSL: SmartAPI returned no candle data for token 14304: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:58.088268+00:00</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>GALLANTT: SmartAPI returned no candle data for token 13337: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:58.779806+00:00</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>GICRE: SmartAPI returned no candle data for token 277: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:30:59.530495+00:00</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>GLAND: SmartAPI returned no candle data for token 1186: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:00.252136+00:00</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>GLENMARK: SmartAPI returned no candle data for token 7406: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:00.964269+00:00</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>GMDCLTD: SmartAPI returned no candle data for token 5204: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:01.650704+00:00</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>GODFRYPHLP: SmartAPI returned no candle data for token 1181: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:02.371911+00:00</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>GODREJCP: SmartAPI returned no candle data for token 10099: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:03.083058+00:00</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>GODREJIND: SmartAPI returned no candle data for token 10925: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:03.760689+00:00</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>GODREJPROP: SmartAPI returned no candle data for token 17875: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:04.455768+00:00</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>GPIL: SmartAPI returned no candle data for token 13409: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:05.175913+00:00</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>GRASIM: SmartAPI returned no candle data for token 1232: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:05.860456+00:00</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>GRSE: SmartAPI returned no candle data for token 5475: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:06.583323+00:00</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>HDBFS: SmartAPI returned no candle data for token 757772: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:07.272041+00:00</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>HDFCLIFE: SmartAPI returned no candle data for token 467: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:07.960078+00:00</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>HINDALCO: SmartAPI returned no candle data for token 1363: Invalid Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:31:08.682968+00:00</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>CANDLE_FETCH_FAILED</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>HINDCOPPER: SmartAPI returned no candle data for token 17939: Invalid Token</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D178"/>
+  <autoFilter ref="A1:D275"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>